<commit_message>
Import and export templates
</commit_message>
<xml_diff>
--- a/examples/sample_providers.xlsx
+++ b/examples/sample_providers.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,11 +439,6 @@
           <t>notes</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>is_active</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -456,9 +451,6 @@
           <t>Primary provider for GPT models.</t>
         </is>
       </c>
-      <c r="C2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -471,9 +463,6 @@
           <t>Provider for Claude model family.</t>
         </is>
       </c>
-      <c r="C3" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -485,9 +474,6 @@
         <is>
           <t>Internal Azure AI Foundry integration.</t>
         </is>
-      </c>
-      <c r="C4" t="b">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>